<commit_message>
Add configurable legend settings to All Profiles View
- Add LEGEND_LOCATIONS and LEGEND_MODES constants
- Add Legend collapsible group in settings panel (mode, position,
  font size, columns, transparency, frame toggle)
- Replace all 9 hard-coded legend calls with _apply_legend() helper
- Summary mode shows only Median/stats, Compact mode auto-adjusts
- Thread legend_cfg through save_publication, save_profiles, save_combined
- All 149 tests pass

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/hvstrip_progressive/Example/Multi_files/sample_input/Profile_10.xlsx
+++ b/hvstrip_progressive/Example/Multi_files/sample_input/Profile_10.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Runs\Readfield\Proccessed\Dinver_3\Redfield_extra\Final_table\profiles_Input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Narm_Afzar\Git_hub\HV_Pro\HV_Analyze_Pro\hvsr_pro\packages\hvstrip-progressive\hvstrip_progressive\Example\Multi_files\sample_input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62709430-0BF4-43B5-963B-0EEADE6B59F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C73EFFE0-5A33-4B61-A34C-506A47619186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="525" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -378,7 +378,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -411,10 +411,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>0</v>
+        <v>2.1335999999999999</v>
       </c>
       <c r="B3">
-        <v>161.54400000000001</v>
+        <v>332.23200000000003</v>
       </c>
       <c r="C3">
         <v>1700</v>
@@ -425,7 +425,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>2.1335999999999999</v>
+        <v>4.8768000000000002</v>
       </c>
       <c r="B4">
         <v>332.23200000000003</v>
@@ -439,10 +439,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>4.8768000000000002</v>
+        <v>15.849600000000001</v>
       </c>
       <c r="B5">
-        <v>332.23200000000003</v>
+        <v>384.048</v>
       </c>
       <c r="C5">
         <v>1700</v>
@@ -453,10 +453,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>15.849600000000001</v>
+        <v>7.1196403200000011</v>
       </c>
       <c r="B6">
-        <v>384.048</v>
+        <v>464.82000000000005</v>
       </c>
       <c r="C6">
         <v>1700</v>
@@ -467,10 +467,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>7.1196403200000011</v>
+        <v>6.9011596799999992</v>
       </c>
       <c r="B7">
-        <v>464.82000000000005</v>
+        <v>487.39044000000001</v>
       </c>
       <c r="C7">
         <v>1700</v>
@@ -481,7 +481,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>6.9011596799999992</v>
+        <v>39.481780319999991</v>
       </c>
       <c r="B8">
         <v>487.39044000000001</v>
@@ -495,10 +495,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>39.481780319999991</v>
+        <v>68.481305760000012</v>
       </c>
       <c r="B9">
-        <v>487.39044000000001</v>
+        <v>649.13256000000001</v>
       </c>
       <c r="C9">
         <v>1700</v>
@@ -509,24 +509,24 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>68.481305760000012</v>
+        <v>28.338170399999989</v>
       </c>
       <c r="B10">
-        <v>649.13256000000001</v>
+        <v>739.50271200000009</v>
       </c>
       <c r="C10">
         <v>1700</v>
       </c>
       <c r="D10">
-        <v>1800</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>28.338170399999989</v>
+        <v>125.78358384000001</v>
       </c>
       <c r="B11">
-        <v>739.50271200000009</v>
+        <v>770.96112000000005</v>
       </c>
       <c r="C11">
         <v>1700</v>
@@ -537,10 +537,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>125.78358384000001</v>
+        <v>194.08837992000002</v>
       </c>
       <c r="B12">
-        <v>770.96112000000005</v>
+        <v>831.13473600000009</v>
       </c>
       <c r="C12">
         <v>1700</v>
@@ -551,13 +551,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>194.08837992000002</v>
+        <v>305.94741959999993</v>
       </c>
       <c r="B13">
-        <v>831.13473600000009</v>
+        <v>897.64819199999999</v>
       </c>
       <c r="C13">
-        <v>1700</v>
+        <v>1795.296384</v>
       </c>
       <c r="D13">
         <v>2000</v>
@@ -565,29 +565,15 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>305.94741959999993</v>
+        <v>0</v>
       </c>
       <c r="B14">
-        <v>897.64819199999999</v>
+        <v>1833.9602640000003</v>
       </c>
       <c r="C14">
-        <v>1795.296384</v>
+        <v>3667.9205280000006</v>
       </c>
       <c r="D14">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>0</v>
-      </c>
-      <c r="B15">
-        <v>1833.9602640000003</v>
-      </c>
-      <c r="C15">
-        <v>3667.9205280000006</v>
-      </c>
-      <c r="D15">
         <v>2000</v>
       </c>
     </row>

</xml_diff>